<commit_message>
SPM-29: new test cases
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-29_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-29_Test_Cases.xlsx
@@ -12,6 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC03" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC04" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC05" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC06" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC07" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -451,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -670,82 +672,148 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>TC06</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>SPM-29-TC06</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>The smallest request is accepted: exactly one item and a one-character message, saved without surrounding spaces</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>AC1, AC2</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>Boundary</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>TC07</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>SPM-29-TC07</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>A clarification request appears only on the event it was sent for, not on another event of the same organiser</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>AC4</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>AC</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Acceptance Criterion</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="9" t="n"/>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>Covered by</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="n"/>
-    </row>
-    <row r="12" ht="31" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>AC1</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>The Event Coordinator can identify which information requires clarification.</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="n"/>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="11" t="inlineStr">
-        <is>
-          <t>SPM-29-TC01
-SPM-29-TC02</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="n"/>
-    </row>
-    <row r="13" ht="31" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>AC2</t>
-        </is>
-      </c>
-      <c r="B13" s="11" t="inlineStr">
-        <is>
-          <t>The Event Coordinator can provide a clarification message.</t>
         </is>
       </c>
       <c r="C13" s="8" t="n"/>
       <c r="D13" s="9" t="n"/>
-      <c r="E13" s="11" t="inlineStr">
-        <is>
-          <t>SPM-29-TC01
-SPM-29-TC02</t>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Covered by</t>
         </is>
       </c>
       <c r="F13" s="9" t="n"/>
     </row>
-    <row r="14" ht="58" customHeight="1">
+    <row r="14" ht="44.5" customHeight="1">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>AC3</t>
+          <t>AC1</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>The event stays Under review while the clarification is open; there is no separate Clarification Required status. The open clarification is shown on the event to the Event Organiser and the assigned Event Coordinator.</t>
+          <t>The Event Coordinator can identify which information requires clarification.</t>
         </is>
       </c>
       <c r="C14" s="8" t="n"/>
       <c r="D14" s="9" t="n"/>
       <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>SPM-29-TC01
+SPM-29-TC02
+SPM-29-TC06</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="n"/>
+    </row>
+    <row r="15" ht="44.5" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>AC2</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>The Event Coordinator can provide a clarification message.</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="9" t="n"/>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>SPM-29-TC01
+SPM-29-TC02
+SPM-29-TC06</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="n"/>
+    </row>
+    <row r="16" ht="58" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>AC3</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>The event stays Under review while the clarification is open; there is no separate Clarification Required status. The open clarification is shown on the event to the Event Organiser and the assigned Event Coordinator.</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="9" t="n"/>
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>SPM-29-TC02
 SPM-29-TC03
@@ -753,42 +821,43 @@
 SPM-29-TC05</t>
         </is>
       </c>
-      <c r="F14" s="9" t="n"/>
-    </row>
-    <row r="15" ht="31" customHeight="1">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="F16" s="9" t="n"/>
+    </row>
+    <row r="17" ht="44.5" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>AC4</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>The clarification request is associated with the relevant event.</t>
         </is>
       </c>
-      <c r="C15" s="8" t="n"/>
-      <c r="D15" s="9" t="n"/>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="11" t="inlineStr">
         <is>
           <t>SPM-29-TC02
-SPM-29-TC03</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="n"/>
+SPM-29-TC03
+SPM-29-TC07</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="E12:F12"/>
     <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="E16:F16"/>
     <mergeCell ref="E15:F15"/>
-    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="B17:D17"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="B1:F1"/>
-    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="B16:D16"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
@@ -796,6 +865,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1230,7 +1301,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="58" customHeight="1">
+    <row r="5" ht="31" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1239,12 +1310,11 @@
       <c r="B5" s="13" t="inlineStr">
         <is>
           <t>1. Click 'My Events' in the sidebar
-2. Open 'SPM29 Meridian Open Question Forum'
-3. Go back to My Events and open 'SPM29 Meridian Clarity Summit'</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="71.5" customHeight="1">
+2. Open 'SPM29 Meridian Open Question Forum'</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -1252,13 +1322,12 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Event with an open clarification: SPM29 Meridian Open Question Forum
-Event without one: SPM29 Meridian Clarity Summit
+          <t>Event: SPM29 Meridian Open Question Forum
 Message: Is this a dinner or a conference? Which day do you need?</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="139" customHeight="1">
+    <row r="7" ht="112" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1267,8 +1336,7 @@
       <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Step 1: 'SPM29 Meridian Open Question Forum' is listed with the 'Under review' badge; no 'Clarification required' status appears anywhere.
-Step 2: The event page shows the 'Under review' badge and an amber 'Clarification requested' banner listing 'Purpose, When', the message 'Is this a dinner or a conference? Which day do you need?' and 'Asked by Daniel Tan on 12 Oct 2026, 10:00'.
-Step 3: No 'Clarification requested' banner is shown on 'SPM29 Meridian Clarity Summit'.</t>
+Step 2: The event page shows the 'Under review' badge and an amber 'Clarification requested' banner listing 'Purpose, When', the message 'Is this a dinner or a conference? Which day do you need?' and 'Asked by Daniel Tan on 12 Oct 2026, 10:00'.</t>
         </is>
       </c>
     </row>
@@ -1691,4 +1759,356 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-29-TC06</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="31" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>The smallest request is accepted: exactly one item and a one-character message, saved without surrounding spaces</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="98.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Run `npm run fixtures:spm29` before this case: it sends a request on 'SPM29 Meridian Clarity Summit'. Go straight on to SPM-29-TC07 and reset after that one.
+'SPM29 Meridian Clarity Summit' is Under review, assigned to Daniel Tan, with no clarification open.
+Logged in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="98.5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Click 'Review Queue' in the sidebar and open 'SPM29 Meridian Clarity Summit'
+2. Click 'Review request'
+3. Choose 'Ask the organiser for clarification'
+4. Tick only 'Equipment' under 'What needs clarification'
+5. Type the message in 'Message to the organiser'
+6. Click 'Send request'</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Event: SPM29 Meridian Clarity Summit
+Item: Equipment only (the last item in the list)
+Message: '  ?  ' (a question mark with two spaces before and after it)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="71.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 6: A green 'Clarification requested' message is shown and the status badge still reads 'Under review'. The 'Open clarification' box shows 'Needs clarification: Equipment', the message '?' with no spaces around it, and 'Asked by Daniel Tan' with today's date and time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46314</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-29-TC07</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="31" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>A clarification request appears only on the event it was sent for, not on another event of the same organiser</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="98.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>SPM-29-TC06 has just been run ('SPM29 Meridian Clarity Summit' has an open clarification about Equipment, message '?'). Run `npm run fixtures:spm29` after this case.
+'SPM29 Meridian Open Question Forum' has its own open clarification about Purpose and When.
+Logged in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123), who raised both events.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Click 'My Events' in the sidebar and open 'SPM29 Meridian Open Question Forum'
+2. Go back to My Events and open 'SPM29 Meridian Clarity Summit'</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="71.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Event the request was sent on: SPM29 Meridian Clarity Summit (Equipment, '?')
+Other event: SPM29 Meridian Open Question Forum (Purpose, When, 'Is this a dinner or a conference? Which day do you need?')</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="98.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 1: The 'Clarification requested' banner shows only this event's own clarification: 'Purpose, When' and 'Is this a dinner or a conference? Which day do you need?'. 'Equipment' and '?' do not appear.
+Step 2: The 'Clarification requested' banner shows 'Needs clarification: Equipment' and the message '?', and not the Open Question Forum's items or message.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46314</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>